<commit_message>
data > xl > ml-4350-notes-CY25-Q3a.xlsx: review notation of various authors for spectrum, periododgram, etc.
</commit_message>
<xml_diff>
--- a/data/xl/ml-4350-notes-CY25-Q3a.xlsx
+++ b/data/xl/ml-4350-notes-CY25-Q3a.xlsx
@@ -1,47 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="307" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CDF79F9-A6FF-4FAE-B8D6-5E1689BB3D9D}"/>
+  <xr:revisionPtr revIDLastSave="350" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A24934D8-4E3C-431D-A2EB-D2C63CE03641}"/>
   <bookViews>
-    <workbookView xWindow="3648" yWindow="396" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="786" yWindow="138" windowWidth="18858" windowHeight="11136" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
     <sheet name="eda_sessions" sheetId="10" r:id="rId2"/>
     <sheet name="eda_requests" sheetId="9" r:id="rId3"/>
     <sheet name="fn_sessions" sheetId="8" r:id="rId4"/>
-    <sheet name="toc_292" sheetId="7" r:id="rId5"/>
-    <sheet name="notes_01" sheetId="4" r:id="rId6"/>
-    <sheet name="notes_02" sheetId="5" r:id="rId7"/>
-    <sheet name="notes_03" sheetId="6" r:id="rId8"/>
-    <sheet name="templates" sheetId="1" r:id="rId9"/>
+    <sheet name="fourier_notes" sheetId="11" r:id="rId5"/>
+    <sheet name="toc_292" sheetId="7" r:id="rId6"/>
+    <sheet name="notes_01" sheetId="4" r:id="rId7"/>
+    <sheet name="notes_02" sheetId="5" r:id="rId8"/>
+    <sheet name="notes_03" sheetId="6" r:id="rId9"/>
+    <sheet name="templates" sheetId="1" r:id="rId10"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
+    <externalReference r:id="rId12"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">templates!$B$5:$O$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">toc_292!$B$5:$D$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">templates!$B$5:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">toc_292!$B$5:$D$234</definedName>
     <definedName name="all_Buyers">[1]pct_per_factor!$D$1:$D$65536</definedName>
     <definedName name="corr">[2]statistics!$A$2</definedName>
     <definedName name="noOct">[1]pct_per_factor!$A$6:$IV$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">eda_requests!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">eda_sessions!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">fn_sessions!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">fourier_notes!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">index!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">notes_01!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">notes_02!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">notes_03!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">templates!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">toc_292!$A:$A,toc_292!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">notes_01!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">notes_02!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">notes_03!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">templates!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">toc_292!$A:$A,toc_292!$1:$1</definedName>
     <definedName name="yesOct">[1]pct_per_factor!$A$7:$IV$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -65,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="466">
   <si>
     <t>tag</t>
   </si>
@@ -1379,6 +1381,90 @@
   </si>
   <si>
     <t>ref</t>
+  </si>
+  <si>
+    <t>fourier_notes</t>
+  </si>
+  <si>
+    <t>spectrun notation of various authors</t>
+  </si>
+  <si>
+    <t>key</t>
+  </si>
+  <si>
+    <t>FATS</t>
+  </si>
+  <si>
+    <t>TSDAT</t>
+  </si>
+  <si>
+    <t>TSA5</t>
+  </si>
+  <si>
+    <t>VSCTSA</t>
+  </si>
+  <si>
+    <t>Stat_153</t>
+  </si>
+  <si>
+    <t>spectrum density function</t>
+  </si>
+  <si>
+    <t>spec-dens</t>
+  </si>
+  <si>
+    <t>spec-cum</t>
+  </si>
+  <si>
+    <t>cumulative spectrum funtion</t>
+  </si>
+  <si>
+    <t>f_a_b</t>
+  </si>
+  <si>
+    <t>DFT</t>
+  </si>
+  <si>
+    <t>discrete Fourier transform</t>
+  </si>
+  <si>
+    <t>d_X^(T)</t>
+  </si>
+  <si>
+    <t>periodogram</t>
+  </si>
+  <si>
+    <t>F_a_b</t>
+  </si>
+  <si>
+    <t>cum-DFT</t>
+  </si>
+  <si>
+    <t>cumulative integral of the DFT</t>
+  </si>
+  <si>
+    <t>Z_X^(T)</t>
+  </si>
+  <si>
+    <t>spec-measure</t>
+  </si>
+  <si>
+    <t>spectral measure</t>
+  </si>
+  <si>
+    <t>Z_X</t>
+  </si>
+  <si>
+    <t>I_XX^(T)</t>
+  </si>
+  <si>
+    <t>P_x</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>I</t>
   </si>
 </sst>
 </file>
@@ -1827,6 +1913,10 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2090,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -2223,55 +2313,55 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="44" customFormat="1" ht="12.9" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="44" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D9" s="49">
+        <v>45848</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="44" customFormat="1" ht="12.9" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="44" t="s">
         <v>313</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C10" s="44" t="s">
         <v>314</v>
       </c>
-      <c r="D9" s="48">
+      <c r="D10" s="48">
         <v>45696</v>
       </c>
-      <c r="G9" s="48">
+      <c r="G10" s="48">
         <v>45635</v>
       </c>
-      <c r="H9" s="44" t="s">
+      <c r="H10" s="44" t="s">
         <v>315</v>
       </c>
-      <c r="I9" s="44" t="s">
+      <c r="I10" s="44" t="s">
         <v>316</v>
       </c>
-      <c r="J9" s="44" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="B10" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="30">
-        <v>45698</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="44" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D11" s="30">
         <v>45698</v>
@@ -2288,13 +2378,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12" s="30">
-        <v>45704</v>
+        <v>45698</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>43</v>
@@ -2308,13 +2398,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D13" s="30">
-        <v>45698</v>
+        <v>45704</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>43</v>
@@ -2323,6 +2413,26 @@
         <v>44</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="30">
+        <v>45698</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2332,6 +2442,1022 @@
   <headerFooter>
     <oddHeader>&amp;L&amp;F&amp;CUNCLASSIFIED&amp;R&amp;A</oddHeader>
     <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="15.68359375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.15625" style="1"/>
+    <col min="3" max="3" width="9.15625" style="5"/>
+    <col min="4" max="4" width="9.15625" style="9"/>
+    <col min="5" max="5" width="9.15625" style="12"/>
+    <col min="6" max="6" width="9.15625" style="15"/>
+    <col min="7" max="7" width="9.15625" style="17"/>
+    <col min="8" max="8" width="9.15625" style="21"/>
+    <col min="9" max="9" width="9.68359375" style="24" customWidth="1"/>
+    <col min="10" max="10" width="12.68359375" style="27" customWidth="1"/>
+    <col min="11" max="11" width="15.68359375" style="30" customWidth="1"/>
+    <col min="12" max="12" width="9.68359375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.26171875" style="33" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.68359375" style="36" customWidth="1"/>
+    <col min="15" max="15" width="27.68359375" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.15625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="4">
+        <f xml:space="preserve"> MAX(C$6:C$105)</f>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:I2" si="0" xml:space="preserve"> MAX(D$6:D$105)</f>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="E2" s="11">
+        <f t="shared" si="0"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="F2" s="14">
+        <f t="shared" si="0"/>
+        <v>698.97000433601886</v>
+      </c>
+      <c r="G2" s="16">
+        <f t="shared" si="0"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="H2" s="20">
+        <f t="shared" si="0"/>
+        <v>698.97000433601886</v>
+      </c>
+      <c r="I2" s="23">
+        <f t="shared" si="0"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="J2" s="26"/>
+      <c r="K2" s="29"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="35"/>
+    </row>
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="4">
+        <f xml:space="preserve"> MEDIAN(C$6:C$105)</f>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="D3" s="8">
+        <f t="shared" ref="D3:I3" si="1" xml:space="preserve"> MEDIAN(D$6:D$105)</f>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="E3" s="11">
+        <f t="shared" si="1"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="F3" s="14">
+        <f t="shared" si="1"/>
+        <v>367.87944117144235</v>
+      </c>
+      <c r="G3" s="16">
+        <f t="shared" si="1"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="H3" s="20">
+        <f t="shared" si="1"/>
+        <v>367.87944117144235</v>
+      </c>
+      <c r="I3" s="23">
+        <f t="shared" si="1"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="J3" s="26"/>
+      <c r="K3" s="29"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="35"/>
+    </row>
+    <row r="4" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="4">
+        <f xml:space="preserve"> MIN(C$6:C$105)</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="8">
+        <f t="shared" ref="D4:I4" si="2" xml:space="preserve"> MIN(D$6:D$105)</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G4" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H4" s="20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I4" s="23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="26"/>
+      <c r="K4" s="29"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="35"/>
+    </row>
+    <row r="5" spans="1:15" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="6">
+        <f xml:space="preserve"> COUNTIF(B$6:B$105, TRUE)</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="14">
+        <f xml:space="preserve"> COUNTA(F$6:F$105)</f>
+        <v>15</v>
+      </c>
+      <c r="G5" s="16"/>
+      <c r="H5" s="20">
+        <f xml:space="preserve"> SUM(H$6:H$105)</f>
+        <v>5266.2861589927443</v>
+      </c>
+      <c r="I5" s="23"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="29"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="35"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5">
+        <f xml:space="preserve"> 0</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="9">
+        <f xml:space="preserve"> $C6</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="12">
+        <f xml:space="preserve"> $C6</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="15">
+        <f xml:space="preserve"> 1000 * $C6</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="17">
+        <f xml:space="preserve"> $C6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="21">
+        <f xml:space="preserve"> 1000 * $C6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="24">
+        <f xml:space="preserve"> $C6</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="27">
+        <f xml:space="preserve"> DATE(2001, 1, 1)</f>
+        <v>36892</v>
+      </c>
+      <c r="K6" s="30">
+        <f xml:space="preserve"> DATE(2001, 1, 1)</f>
+        <v>36892</v>
+      </c>
+      <c r="L6" s="1" t="str">
+        <f xml:space="preserve"> CHOOSE(WEEKDAY($J6), "Sun", "Mon", "Tue", "Wed", "Thu", "Fri", "Sat")</f>
+        <v>Mon</v>
+      </c>
+      <c r="M6" s="33">
+        <f xml:space="preserve"> TIME($C6, $C6, $C6)</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="5">
+        <f xml:space="preserve"> EXP(-3)</f>
+        <v>4.9787068367863944E-2</v>
+      </c>
+      <c r="D7" s="9">
+        <f t="shared" ref="D7:I20" si="3" xml:space="preserve"> $C7</f>
+        <v>4.9787068367863944E-2</v>
+      </c>
+      <c r="E7" s="12">
+        <f t="shared" si="3"/>
+        <v>4.9787068367863944E-2</v>
+      </c>
+      <c r="F7" s="15">
+        <f t="shared" ref="F7:H20" si="4" xml:space="preserve"> 1000 * $C7</f>
+        <v>49.787068367863945</v>
+      </c>
+      <c r="G7" s="17">
+        <f t="shared" si="3"/>
+        <v>4.9787068367863944E-2</v>
+      </c>
+      <c r="H7" s="21">
+        <f t="shared" si="4"/>
+        <v>49.787068367863945</v>
+      </c>
+      <c r="I7" s="24">
+        <f t="shared" si="3"/>
+        <v>4.9787068367863944E-2</v>
+      </c>
+      <c r="J7" s="27">
+        <f xml:space="preserve"> DATE(2001 + $C7, 1 + $C7 * 12, 1 + $C7 * 30)</f>
+        <v>36893</v>
+      </c>
+      <c r="K7" s="30">
+        <f xml:space="preserve"> DATE(2001 + $C7, 1 + $C7 * 12, 1 + $C7 * 30)</f>
+        <v>36893</v>
+      </c>
+      <c r="L7" s="1" t="str">
+        <f t="shared" ref="L7:L20" si="5" xml:space="preserve"> CHOOSE(WEEKDAY($J7), "Sun", "Mon", "Tue", "Wed", "Thu", "Fri", "Sat")</f>
+        <v>Tue</v>
+      </c>
+      <c r="M7" s="33">
+        <f t="shared" ref="M7:M20" si="6" xml:space="preserve"> TIME($C7, $C7, $C7)</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="5">
+        <f xml:space="preserve"> 1/11</f>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="D8" s="9">
+        <f t="shared" si="3"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="E8" s="12">
+        <f t="shared" si="3"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="F8" s="15">
+        <f t="shared" si="4"/>
+        <v>90.909090909090907</v>
+      </c>
+      <c r="G8" s="17">
+        <f t="shared" si="3"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="H8" s="21">
+        <f t="shared" si="4"/>
+        <v>90.909090909090907</v>
+      </c>
+      <c r="I8" s="24">
+        <f t="shared" si="3"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="J8" s="27">
+        <f t="shared" ref="J8:K20" si="7" xml:space="preserve"> DATE(2001 + $C8, 1 + $C8 * 12, 1 + $C8 * 30)</f>
+        <v>36925</v>
+      </c>
+      <c r="K8" s="30">
+        <f t="shared" si="7"/>
+        <v>36925</v>
+      </c>
+      <c r="L8" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Sat</v>
+      </c>
+      <c r="M8" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N8" s="36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="5">
+        <f xml:space="preserve"> EXP(-2)</f>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="D9" s="9">
+        <f t="shared" si="3"/>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="E9" s="12">
+        <f t="shared" si="3"/>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="F9" s="15">
+        <f t="shared" si="4"/>
+        <v>135.3352832366127</v>
+      </c>
+      <c r="G9" s="17">
+        <f t="shared" si="3"/>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="H9" s="21">
+        <f t="shared" si="4"/>
+        <v>135.3352832366127</v>
+      </c>
+      <c r="I9" s="24">
+        <f t="shared" si="3"/>
+        <v>0.1353352832366127</v>
+      </c>
+      <c r="J9" s="27">
+        <f t="shared" si="7"/>
+        <v>36927</v>
+      </c>
+      <c r="K9" s="30">
+        <f t="shared" si="7"/>
+        <v>36927</v>
+      </c>
+      <c r="L9" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Mon</v>
+      </c>
+      <c r="M9" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N9" s="36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="5">
+        <f xml:space="preserve"> 1/(2 * PI())</f>
+        <v>0.15915494309189535</v>
+      </c>
+      <c r="D10" s="9">
+        <f t="shared" si="3"/>
+        <v>0.15915494309189535</v>
+      </c>
+      <c r="E10" s="12">
+        <f t="shared" si="3"/>
+        <v>0.15915494309189535</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="4"/>
+        <v>159.15494309189535</v>
+      </c>
+      <c r="G10" s="17">
+        <f t="shared" si="3"/>
+        <v>0.15915494309189535</v>
+      </c>
+      <c r="H10" s="21">
+        <f t="shared" si="4"/>
+        <v>159.15494309189535</v>
+      </c>
+      <c r="I10" s="24">
+        <f t="shared" si="3"/>
+        <v>0.15915494309189535</v>
+      </c>
+      <c r="J10" s="27">
+        <f t="shared" si="7"/>
+        <v>36927</v>
+      </c>
+      <c r="K10" s="30">
+        <f t="shared" si="7"/>
+        <v>36927</v>
+      </c>
+      <c r="L10" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Mon</v>
+      </c>
+      <c r="M10" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N10" s="36" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="1" t="b">
+        <f xml:space="preserve"> TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="C11" s="5">
+        <f>LOG10(2)</f>
+        <v>0.3010299956639812</v>
+      </c>
+      <c r="D11" s="9">
+        <f t="shared" si="3"/>
+        <v>0.3010299956639812</v>
+      </c>
+      <c r="E11" s="12">
+        <f t="shared" si="3"/>
+        <v>0.3010299956639812</v>
+      </c>
+      <c r="F11" s="15">
+        <f t="shared" si="4"/>
+        <v>301.0299956639812</v>
+      </c>
+      <c r="G11" s="17">
+        <f t="shared" si="3"/>
+        <v>0.3010299956639812</v>
+      </c>
+      <c r="H11" s="21">
+        <f t="shared" si="4"/>
+        <v>301.0299956639812</v>
+      </c>
+      <c r="I11" s="24">
+        <f t="shared" si="3"/>
+        <v>0.3010299956639812</v>
+      </c>
+      <c r="J11" s="27">
+        <f t="shared" si="7"/>
+        <v>36991</v>
+      </c>
+      <c r="K11" s="30">
+        <f t="shared" si="7"/>
+        <v>36991</v>
+      </c>
+      <c r="L11" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Tue</v>
+      </c>
+      <c r="M11" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N11" s="36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="5">
+        <f xml:space="preserve"> 1/PI()</f>
+        <v>0.31830988618379069</v>
+      </c>
+      <c r="D12" s="9">
+        <f t="shared" si="3"/>
+        <v>0.31830988618379069</v>
+      </c>
+      <c r="E12" s="12">
+        <f t="shared" si="3"/>
+        <v>0.31830988618379069</v>
+      </c>
+      <c r="F12" s="15">
+        <f t="shared" si="4"/>
+        <v>318.3098861837907</v>
+      </c>
+      <c r="G12" s="17">
+        <f t="shared" si="3"/>
+        <v>0.31830988618379069</v>
+      </c>
+      <c r="H12" s="21">
+        <f t="shared" si="4"/>
+        <v>318.3098861837907</v>
+      </c>
+      <c r="I12" s="24">
+        <f t="shared" si="3"/>
+        <v>0.31830988618379069</v>
+      </c>
+      <c r="J12" s="27">
+        <f t="shared" si="7"/>
+        <v>36991</v>
+      </c>
+      <c r="K12" s="30">
+        <f t="shared" si="7"/>
+        <v>36991</v>
+      </c>
+      <c r="L12" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Tue</v>
+      </c>
+      <c r="M12" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N12" s="36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="5">
+        <f xml:space="preserve"> EXP(-1)</f>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="D13" s="9">
+        <f t="shared" si="3"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="E13" s="12">
+        <f t="shared" si="3"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="F13" s="15">
+        <f t="shared" si="4"/>
+        <v>367.87944117144235</v>
+      </c>
+      <c r="G13" s="17">
+        <f t="shared" si="3"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="H13" s="21">
+        <f t="shared" si="4"/>
+        <v>367.87944117144235</v>
+      </c>
+      <c r="I13" s="24">
+        <f t="shared" si="3"/>
+        <v>0.36787944117144233</v>
+      </c>
+      <c r="J13" s="27">
+        <f t="shared" si="7"/>
+        <v>37023</v>
+      </c>
+      <c r="K13" s="30">
+        <f t="shared" si="7"/>
+        <v>37023</v>
+      </c>
+      <c r="L13" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Sat</v>
+      </c>
+      <c r="M13" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N13" s="36" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="5">
+        <f xml:space="preserve"> (2 * PI())^(-1/2)</f>
+        <v>0.3989422804014327</v>
+      </c>
+      <c r="D14" s="9">
+        <f t="shared" si="3"/>
+        <v>0.3989422804014327</v>
+      </c>
+      <c r="E14" s="12">
+        <f t="shared" si="3"/>
+        <v>0.3989422804014327</v>
+      </c>
+      <c r="F14" s="15">
+        <f t="shared" si="4"/>
+        <v>398.9422804014327</v>
+      </c>
+      <c r="G14" s="17">
+        <f t="shared" si="3"/>
+        <v>0.3989422804014327</v>
+      </c>
+      <c r="H14" s="21">
+        <f t="shared" si="4"/>
+        <v>398.9422804014327</v>
+      </c>
+      <c r="I14" s="24">
+        <f t="shared" si="3"/>
+        <v>0.3989422804014327</v>
+      </c>
+      <c r="J14" s="27">
+        <f t="shared" si="7"/>
+        <v>37023</v>
+      </c>
+      <c r="K14" s="30">
+        <f t="shared" si="7"/>
+        <v>37023</v>
+      </c>
+      <c r="L14" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Sat</v>
+      </c>
+      <c r="M14" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="36" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="5">
+        <f>LOG10(EXP(1))</f>
+        <v>0.43429448190325182</v>
+      </c>
+      <c r="D15" s="9">
+        <f t="shared" si="3"/>
+        <v>0.43429448190325182</v>
+      </c>
+      <c r="E15" s="12">
+        <f t="shared" si="3"/>
+        <v>0.43429448190325182</v>
+      </c>
+      <c r="F15" s="15">
+        <f t="shared" si="4"/>
+        <v>434.29448190325184</v>
+      </c>
+      <c r="G15" s="17">
+        <f t="shared" si="3"/>
+        <v>0.43429448190325182</v>
+      </c>
+      <c r="H15" s="21">
+        <f t="shared" si="4"/>
+        <v>434.29448190325184</v>
+      </c>
+      <c r="I15" s="24">
+        <f t="shared" si="3"/>
+        <v>0.43429448190325182</v>
+      </c>
+      <c r="J15" s="27">
+        <f t="shared" si="7"/>
+        <v>37056</v>
+      </c>
+      <c r="K15" s="30">
+        <f t="shared" si="7"/>
+        <v>37056</v>
+      </c>
+      <c r="L15" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Thu</v>
+      </c>
+      <c r="M15" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N15" s="36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="1" t="b">
+        <f xml:space="preserve"> TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="C16" s="5">
+        <f>LOG10(3)</f>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="D16" s="9">
+        <f t="shared" si="3"/>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="E16" s="12">
+        <f t="shared" si="3"/>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="F16" s="15">
+        <f t="shared" si="4"/>
+        <v>477.12125471966243</v>
+      </c>
+      <c r="G16" s="17">
+        <f t="shared" si="3"/>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="H16" s="21">
+        <f t="shared" si="4"/>
+        <v>477.12125471966243</v>
+      </c>
+      <c r="I16" s="24">
+        <f t="shared" si="3"/>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="J16" s="27">
+        <f t="shared" si="7"/>
+        <v>37057</v>
+      </c>
+      <c r="K16" s="30">
+        <f t="shared" si="7"/>
+        <v>37057</v>
+      </c>
+      <c r="L16" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Fri</v>
+      </c>
+      <c r="M16" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N16" s="36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="5">
+        <f xml:space="preserve"> PI()^(-1/2)</f>
+        <v>0.56418958354775628</v>
+      </c>
+      <c r="D17" s="9">
+        <f t="shared" si="3"/>
+        <v>0.56418958354775628</v>
+      </c>
+      <c r="E17" s="12">
+        <f t="shared" si="3"/>
+        <v>0.56418958354775628</v>
+      </c>
+      <c r="F17" s="15">
+        <f t="shared" si="4"/>
+        <v>564.18958354775623</v>
+      </c>
+      <c r="G17" s="17">
+        <f t="shared" si="3"/>
+        <v>0.56418958354775628</v>
+      </c>
+      <c r="H17" s="21">
+        <f t="shared" si="4"/>
+        <v>564.18958354775623</v>
+      </c>
+      <c r="I17" s="24">
+        <f t="shared" si="3"/>
+        <v>0.56418958354775628</v>
+      </c>
+      <c r="J17" s="27">
+        <f t="shared" si="7"/>
+        <v>37089</v>
+      </c>
+      <c r="K17" s="30">
+        <f t="shared" si="7"/>
+        <v>37089</v>
+      </c>
+      <c r="L17" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Tue</v>
+      </c>
+      <c r="M17" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N17" s="36" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="5">
+        <f xml:space="preserve"> 0.5772156649</f>
+        <v>0.57721566489999998</v>
+      </c>
+      <c r="D18" s="9">
+        <f t="shared" si="3"/>
+        <v>0.57721566489999998</v>
+      </c>
+      <c r="E18" s="12">
+        <f t="shared" si="3"/>
+        <v>0.57721566489999998</v>
+      </c>
+      <c r="F18" s="15">
+        <f t="shared" si="4"/>
+        <v>577.21566489999998</v>
+      </c>
+      <c r="G18" s="17">
+        <f t="shared" si="3"/>
+        <v>0.57721566489999998</v>
+      </c>
+      <c r="H18" s="21">
+        <f t="shared" si="4"/>
+        <v>577.21566489999998</v>
+      </c>
+      <c r="I18" s="24">
+        <f t="shared" si="3"/>
+        <v>0.57721566489999998</v>
+      </c>
+      <c r="J18" s="27">
+        <f t="shared" si="7"/>
+        <v>37090</v>
+      </c>
+      <c r="K18" s="30">
+        <f t="shared" si="7"/>
+        <v>37090</v>
+      </c>
+      <c r="L18" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Wed</v>
+      </c>
+      <c r="M18" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N18" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="5">
+        <f xml:space="preserve"> LN(2)</f>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="D19" s="9">
+        <f t="shared" si="3"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="E19" s="12">
+        <f t="shared" si="3"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="F19" s="15">
+        <f t="shared" si="4"/>
+        <v>693.14718055994524</v>
+      </c>
+      <c r="G19" s="17">
+        <f t="shared" si="3"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="H19" s="21">
+        <f t="shared" si="4"/>
+        <v>693.14718055994524</v>
+      </c>
+      <c r="I19" s="24">
+        <f t="shared" si="3"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="J19" s="27">
+        <f t="shared" si="7"/>
+        <v>37155</v>
+      </c>
+      <c r="K19" s="30">
+        <f t="shared" si="7"/>
+        <v>37155</v>
+      </c>
+      <c r="L19" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Fri</v>
+      </c>
+      <c r="M19" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N19" s="36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="1" t="b">
+        <f xml:space="preserve"> TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="C20" s="5">
+        <f>LOG10(5)</f>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="D20" s="9">
+        <f t="shared" si="3"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="E20" s="12">
+        <f t="shared" si="3"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="F20" s="15">
+        <f t="shared" si="4"/>
+        <v>698.97000433601886</v>
+      </c>
+      <c r="G20" s="17">
+        <f t="shared" si="3"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="H20" s="21">
+        <f t="shared" si="4"/>
+        <v>698.97000433601886</v>
+      </c>
+      <c r="I20" s="24">
+        <f t="shared" si="3"/>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="J20" s="27">
+        <f t="shared" si="7"/>
+        <v>37155</v>
+      </c>
+      <c r="K20" s="30">
+        <f t="shared" si="7"/>
+        <v>37155</v>
+      </c>
+      <c r="L20" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Fri</v>
+      </c>
+      <c r="M20" s="33">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="36" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B5:O5" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;F&amp;CU//FOUO&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;Lprinted: &amp;D&amp;CU//FOUO&amp;Rpage &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -3348,6 +4474,148 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91584213-8A6C-41CA-9D43-C995C5AD5E50}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5234375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.68359375" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.15625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="3" customFormat="1" ht="11.7" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="3" customFormat="1" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C7" s="50" t="s">
+        <v>449</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>452</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="44" customFormat="1" ht="12.9" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="44" t="s">
+        <v>456</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>457</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" s="44" t="s">
+        <v>454</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>454</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;F&amp;CUNCLASSIFIED&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B58712-5292-4A29-B1B7-4787EE57F779}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -6632,7 +7900,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -6779,7 +8047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -6990,7 +8258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -7255,1020 +8523,4 @@
     <oddFooter>&amp;Lprinted: &amp;D&amp;CUNCLASSIFIED&amp;Rpage &amp;P of &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
-  <cols>
-    <col min="1" max="1" width="15.68359375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.15625" style="1"/>
-    <col min="3" max="3" width="9.15625" style="5"/>
-    <col min="4" max="4" width="9.15625" style="9"/>
-    <col min="5" max="5" width="9.15625" style="12"/>
-    <col min="6" max="6" width="9.15625" style="15"/>
-    <col min="7" max="7" width="9.15625" style="17"/>
-    <col min="8" max="8" width="9.15625" style="21"/>
-    <col min="9" max="9" width="9.68359375" style="24" customWidth="1"/>
-    <col min="10" max="10" width="12.68359375" style="27" customWidth="1"/>
-    <col min="11" max="11" width="15.68359375" style="30" customWidth="1"/>
-    <col min="12" max="12" width="9.68359375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.26171875" style="33" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.68359375" style="36" customWidth="1"/>
-    <col min="15" max="15" width="27.68359375" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.15625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="4">
-        <f xml:space="preserve"> MAX(C$6:C$105)</f>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="D2" s="8">
-        <f t="shared" ref="D2:I2" si="0" xml:space="preserve"> MAX(D$6:D$105)</f>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="E2" s="11">
-        <f t="shared" si="0"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="F2" s="14">
-        <f t="shared" si="0"/>
-        <v>698.97000433601886</v>
-      </c>
-      <c r="G2" s="16">
-        <f t="shared" si="0"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="H2" s="20">
-        <f t="shared" si="0"/>
-        <v>698.97000433601886</v>
-      </c>
-      <c r="I2" s="23">
-        <f t="shared" si="0"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="29"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="35"/>
-    </row>
-    <row r="3" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="4">
-        <f xml:space="preserve"> MEDIAN(C$6:C$105)</f>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="D3" s="8">
-        <f t="shared" ref="D3:I3" si="1" xml:space="preserve"> MEDIAN(D$6:D$105)</f>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="E3" s="11">
-        <f t="shared" si="1"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="F3" s="14">
-        <f t="shared" si="1"/>
-        <v>367.87944117144235</v>
-      </c>
-      <c r="G3" s="16">
-        <f t="shared" si="1"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="H3" s="20">
-        <f t="shared" si="1"/>
-        <v>367.87944117144235</v>
-      </c>
-      <c r="I3" s="23">
-        <f t="shared" si="1"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="29"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="35"/>
-    </row>
-    <row r="4" spans="1:15" s="3" customFormat="1" ht="11.7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="4">
-        <f xml:space="preserve"> MIN(C$6:C$105)</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="8">
-        <f t="shared" ref="D4:I4" si="2" xml:space="preserve"> MIN(D$6:D$105)</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="11">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F4" s="14">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G4" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H4" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I4" s="23">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J4" s="26"/>
-      <c r="K4" s="29"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="35"/>
-    </row>
-    <row r="5" spans="1:15" s="3" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="6">
-        <f xml:space="preserve"> COUNTIF(B$6:B$105, TRUE)</f>
-        <v>3</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="14">
-        <f xml:space="preserve"> COUNTA(F$6:F$105)</f>
-        <v>15</v>
-      </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="20">
-        <f xml:space="preserve"> SUM(H$6:H$105)</f>
-        <v>5266.2861589927443</v>
-      </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="29"/>
-      <c r="M5" s="32"/>
-      <c r="N5" s="35"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="5">
-        <f xml:space="preserve"> 0</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="9">
-        <f xml:space="preserve"> $C6</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="12">
-        <f xml:space="preserve"> $C6</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="15">
-        <f xml:space="preserve"> 1000 * $C6</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="17">
-        <f xml:space="preserve"> $C6</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="21">
-        <f xml:space="preserve"> 1000 * $C6</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="24">
-        <f xml:space="preserve"> $C6</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="27">
-        <f xml:space="preserve"> DATE(2001, 1, 1)</f>
-        <v>36892</v>
-      </c>
-      <c r="K6" s="30">
-        <f xml:space="preserve"> DATE(2001, 1, 1)</f>
-        <v>36892</v>
-      </c>
-      <c r="L6" s="1" t="str">
-        <f xml:space="preserve"> CHOOSE(WEEKDAY($J6), "Sun", "Mon", "Tue", "Wed", "Thu", "Fri", "Sat")</f>
-        <v>Mon</v>
-      </c>
-      <c r="M6" s="33">
-        <f xml:space="preserve"> TIME($C6, $C6, $C6)</f>
-        <v>0</v>
-      </c>
-      <c r="N6" s="36" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="5">
-        <f xml:space="preserve"> EXP(-3)</f>
-        <v>4.9787068367863944E-2</v>
-      </c>
-      <c r="D7" s="9">
-        <f t="shared" ref="D7:I20" si="3" xml:space="preserve"> $C7</f>
-        <v>4.9787068367863944E-2</v>
-      </c>
-      <c r="E7" s="12">
-        <f t="shared" si="3"/>
-        <v>4.9787068367863944E-2</v>
-      </c>
-      <c r="F7" s="15">
-        <f t="shared" ref="F7:H20" si="4" xml:space="preserve"> 1000 * $C7</f>
-        <v>49.787068367863945</v>
-      </c>
-      <c r="G7" s="17">
-        <f t="shared" si="3"/>
-        <v>4.9787068367863944E-2</v>
-      </c>
-      <c r="H7" s="21">
-        <f t="shared" si="4"/>
-        <v>49.787068367863945</v>
-      </c>
-      <c r="I7" s="24">
-        <f t="shared" si="3"/>
-        <v>4.9787068367863944E-2</v>
-      </c>
-      <c r="J7" s="27">
-        <f xml:space="preserve"> DATE(2001 + $C7, 1 + $C7 * 12, 1 + $C7 * 30)</f>
-        <v>36893</v>
-      </c>
-      <c r="K7" s="30">
-        <f xml:space="preserve"> DATE(2001 + $C7, 1 + $C7 * 12, 1 + $C7 * 30)</f>
-        <v>36893</v>
-      </c>
-      <c r="L7" s="1" t="str">
-        <f t="shared" ref="L7:L20" si="5" xml:space="preserve"> CHOOSE(WEEKDAY($J7), "Sun", "Mon", "Tue", "Wed", "Thu", "Fri", "Sat")</f>
-        <v>Tue</v>
-      </c>
-      <c r="M7" s="33">
-        <f t="shared" ref="M7:M20" si="6" xml:space="preserve"> TIME($C7, $C7, $C7)</f>
-        <v>0</v>
-      </c>
-      <c r="N7" s="36" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="5">
-        <f xml:space="preserve"> 1/11</f>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="D8" s="9">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="E8" s="12">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="F8" s="15">
-        <f t="shared" si="4"/>
-        <v>90.909090909090907</v>
-      </c>
-      <c r="G8" s="17">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="H8" s="21">
-        <f t="shared" si="4"/>
-        <v>90.909090909090907</v>
-      </c>
-      <c r="I8" s="24">
-        <f t="shared" si="3"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="J8" s="27">
-        <f t="shared" ref="J8:K20" si="7" xml:space="preserve"> DATE(2001 + $C8, 1 + $C8 * 12, 1 + $C8 * 30)</f>
-        <v>36925</v>
-      </c>
-      <c r="K8" s="30">
-        <f t="shared" si="7"/>
-        <v>36925</v>
-      </c>
-      <c r="L8" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Sat</v>
-      </c>
-      <c r="M8" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="5">
-        <f xml:space="preserve"> EXP(-2)</f>
-        <v>0.1353352832366127</v>
-      </c>
-      <c r="D9" s="9">
-        <f t="shared" si="3"/>
-        <v>0.1353352832366127</v>
-      </c>
-      <c r="E9" s="12">
-        <f t="shared" si="3"/>
-        <v>0.1353352832366127</v>
-      </c>
-      <c r="F9" s="15">
-        <f t="shared" si="4"/>
-        <v>135.3352832366127</v>
-      </c>
-      <c r="G9" s="17">
-        <f t="shared" si="3"/>
-        <v>0.1353352832366127</v>
-      </c>
-      <c r="H9" s="21">
-        <f t="shared" si="4"/>
-        <v>135.3352832366127</v>
-      </c>
-      <c r="I9" s="24">
-        <f t="shared" si="3"/>
-        <v>0.1353352832366127</v>
-      </c>
-      <c r="J9" s="27">
-        <f t="shared" si="7"/>
-        <v>36927</v>
-      </c>
-      <c r="K9" s="30">
-        <f t="shared" si="7"/>
-        <v>36927</v>
-      </c>
-      <c r="L9" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Mon</v>
-      </c>
-      <c r="M9" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="36" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="5">
-        <f xml:space="preserve"> 1/(2 * PI())</f>
-        <v>0.15915494309189535</v>
-      </c>
-      <c r="D10" s="9">
-        <f t="shared" si="3"/>
-        <v>0.15915494309189535</v>
-      </c>
-      <c r="E10" s="12">
-        <f t="shared" si="3"/>
-        <v>0.15915494309189535</v>
-      </c>
-      <c r="F10" s="15">
-        <f t="shared" si="4"/>
-        <v>159.15494309189535</v>
-      </c>
-      <c r="G10" s="17">
-        <f t="shared" si="3"/>
-        <v>0.15915494309189535</v>
-      </c>
-      <c r="H10" s="21">
-        <f t="shared" si="4"/>
-        <v>159.15494309189535</v>
-      </c>
-      <c r="I10" s="24">
-        <f t="shared" si="3"/>
-        <v>0.15915494309189535</v>
-      </c>
-      <c r="J10" s="27">
-        <f t="shared" si="7"/>
-        <v>36927</v>
-      </c>
-      <c r="K10" s="30">
-        <f t="shared" si="7"/>
-        <v>36927</v>
-      </c>
-      <c r="L10" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Mon</v>
-      </c>
-      <c r="M10" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N10" s="36" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="1" t="b">
-        <f xml:space="preserve"> TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="5">
-        <f>LOG10(2)</f>
-        <v>0.3010299956639812</v>
-      </c>
-      <c r="D11" s="9">
-        <f t="shared" si="3"/>
-        <v>0.3010299956639812</v>
-      </c>
-      <c r="E11" s="12">
-        <f t="shared" si="3"/>
-        <v>0.3010299956639812</v>
-      </c>
-      <c r="F11" s="15">
-        <f t="shared" si="4"/>
-        <v>301.0299956639812</v>
-      </c>
-      <c r="G11" s="17">
-        <f t="shared" si="3"/>
-        <v>0.3010299956639812</v>
-      </c>
-      <c r="H11" s="21">
-        <f t="shared" si="4"/>
-        <v>301.0299956639812</v>
-      </c>
-      <c r="I11" s="24">
-        <f t="shared" si="3"/>
-        <v>0.3010299956639812</v>
-      </c>
-      <c r="J11" s="27">
-        <f t="shared" si="7"/>
-        <v>36991</v>
-      </c>
-      <c r="K11" s="30">
-        <f t="shared" si="7"/>
-        <v>36991</v>
-      </c>
-      <c r="L11" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Tue</v>
-      </c>
-      <c r="M11" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N11" s="36" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5">
-        <f xml:space="preserve"> 1/PI()</f>
-        <v>0.31830988618379069</v>
-      </c>
-      <c r="D12" s="9">
-        <f t="shared" si="3"/>
-        <v>0.31830988618379069</v>
-      </c>
-      <c r="E12" s="12">
-        <f t="shared" si="3"/>
-        <v>0.31830988618379069</v>
-      </c>
-      <c r="F12" s="15">
-        <f t="shared" si="4"/>
-        <v>318.3098861837907</v>
-      </c>
-      <c r="G12" s="17">
-        <f t="shared" si="3"/>
-        <v>0.31830988618379069</v>
-      </c>
-      <c r="H12" s="21">
-        <f t="shared" si="4"/>
-        <v>318.3098861837907</v>
-      </c>
-      <c r="I12" s="24">
-        <f t="shared" si="3"/>
-        <v>0.31830988618379069</v>
-      </c>
-      <c r="J12" s="27">
-        <f t="shared" si="7"/>
-        <v>36991</v>
-      </c>
-      <c r="K12" s="30">
-        <f t="shared" si="7"/>
-        <v>36991</v>
-      </c>
-      <c r="L12" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Tue</v>
-      </c>
-      <c r="M12" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N12" s="36" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="5">
-        <f xml:space="preserve"> EXP(-1)</f>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="D13" s="9">
-        <f t="shared" si="3"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="E13" s="12">
-        <f t="shared" si="3"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="F13" s="15">
-        <f t="shared" si="4"/>
-        <v>367.87944117144235</v>
-      </c>
-      <c r="G13" s="17">
-        <f t="shared" si="3"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="H13" s="21">
-        <f t="shared" si="4"/>
-        <v>367.87944117144235</v>
-      </c>
-      <c r="I13" s="24">
-        <f t="shared" si="3"/>
-        <v>0.36787944117144233</v>
-      </c>
-      <c r="J13" s="27">
-        <f t="shared" si="7"/>
-        <v>37023</v>
-      </c>
-      <c r="K13" s="30">
-        <f t="shared" si="7"/>
-        <v>37023</v>
-      </c>
-      <c r="L13" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Sat</v>
-      </c>
-      <c r="M13" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N13" s="36" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="5">
-        <f xml:space="preserve"> (2 * PI())^(-1/2)</f>
-        <v>0.3989422804014327</v>
-      </c>
-      <c r="D14" s="9">
-        <f t="shared" si="3"/>
-        <v>0.3989422804014327</v>
-      </c>
-      <c r="E14" s="12">
-        <f t="shared" si="3"/>
-        <v>0.3989422804014327</v>
-      </c>
-      <c r="F14" s="15">
-        <f t="shared" si="4"/>
-        <v>398.9422804014327</v>
-      </c>
-      <c r="G14" s="17">
-        <f t="shared" si="3"/>
-        <v>0.3989422804014327</v>
-      </c>
-      <c r="H14" s="21">
-        <f t="shared" si="4"/>
-        <v>398.9422804014327</v>
-      </c>
-      <c r="I14" s="24">
-        <f t="shared" si="3"/>
-        <v>0.3989422804014327</v>
-      </c>
-      <c r="J14" s="27">
-        <f t="shared" si="7"/>
-        <v>37023</v>
-      </c>
-      <c r="K14" s="30">
-        <f t="shared" si="7"/>
-        <v>37023</v>
-      </c>
-      <c r="L14" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Sat</v>
-      </c>
-      <c r="M14" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N14" s="36" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="5">
-        <f>LOG10(EXP(1))</f>
-        <v>0.43429448190325182</v>
-      </c>
-      <c r="D15" s="9">
-        <f t="shared" si="3"/>
-        <v>0.43429448190325182</v>
-      </c>
-      <c r="E15" s="12">
-        <f t="shared" si="3"/>
-        <v>0.43429448190325182</v>
-      </c>
-      <c r="F15" s="15">
-        <f t="shared" si="4"/>
-        <v>434.29448190325184</v>
-      </c>
-      <c r="G15" s="17">
-        <f t="shared" si="3"/>
-        <v>0.43429448190325182</v>
-      </c>
-      <c r="H15" s="21">
-        <f t="shared" si="4"/>
-        <v>434.29448190325184</v>
-      </c>
-      <c r="I15" s="24">
-        <f t="shared" si="3"/>
-        <v>0.43429448190325182</v>
-      </c>
-      <c r="J15" s="27">
-        <f t="shared" si="7"/>
-        <v>37056</v>
-      </c>
-      <c r="K15" s="30">
-        <f t="shared" si="7"/>
-        <v>37056</v>
-      </c>
-      <c r="L15" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Thu</v>
-      </c>
-      <c r="M15" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N15" s="36" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="1" t="b">
-        <f xml:space="preserve"> TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="C16" s="5">
-        <f>LOG10(3)</f>
-        <v>0.47712125471966244</v>
-      </c>
-      <c r="D16" s="9">
-        <f t="shared" si="3"/>
-        <v>0.47712125471966244</v>
-      </c>
-      <c r="E16" s="12">
-        <f t="shared" si="3"/>
-        <v>0.47712125471966244</v>
-      </c>
-      <c r="F16" s="15">
-        <f t="shared" si="4"/>
-        <v>477.12125471966243</v>
-      </c>
-      <c r="G16" s="17">
-        <f t="shared" si="3"/>
-        <v>0.47712125471966244</v>
-      </c>
-      <c r="H16" s="21">
-        <f t="shared" si="4"/>
-        <v>477.12125471966243</v>
-      </c>
-      <c r="I16" s="24">
-        <f t="shared" si="3"/>
-        <v>0.47712125471966244</v>
-      </c>
-      <c r="J16" s="27">
-        <f t="shared" si="7"/>
-        <v>37057</v>
-      </c>
-      <c r="K16" s="30">
-        <f t="shared" si="7"/>
-        <v>37057</v>
-      </c>
-      <c r="L16" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Fri</v>
-      </c>
-      <c r="M16" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N16" s="36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="5">
-        <f xml:space="preserve"> PI()^(-1/2)</f>
-        <v>0.56418958354775628</v>
-      </c>
-      <c r="D17" s="9">
-        <f t="shared" si="3"/>
-        <v>0.56418958354775628</v>
-      </c>
-      <c r="E17" s="12">
-        <f t="shared" si="3"/>
-        <v>0.56418958354775628</v>
-      </c>
-      <c r="F17" s="15">
-        <f t="shared" si="4"/>
-        <v>564.18958354775623</v>
-      </c>
-      <c r="G17" s="17">
-        <f t="shared" si="3"/>
-        <v>0.56418958354775628</v>
-      </c>
-      <c r="H17" s="21">
-        <f t="shared" si="4"/>
-        <v>564.18958354775623</v>
-      </c>
-      <c r="I17" s="24">
-        <f t="shared" si="3"/>
-        <v>0.56418958354775628</v>
-      </c>
-      <c r="J17" s="27">
-        <f t="shared" si="7"/>
-        <v>37089</v>
-      </c>
-      <c r="K17" s="30">
-        <f t="shared" si="7"/>
-        <v>37089</v>
-      </c>
-      <c r="L17" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Tue</v>
-      </c>
-      <c r="M17" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N17" s="36" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="5">
-        <f xml:space="preserve"> 0.5772156649</f>
-        <v>0.57721566489999998</v>
-      </c>
-      <c r="D18" s="9">
-        <f t="shared" si="3"/>
-        <v>0.57721566489999998</v>
-      </c>
-      <c r="E18" s="12">
-        <f t="shared" si="3"/>
-        <v>0.57721566489999998</v>
-      </c>
-      <c r="F18" s="15">
-        <f t="shared" si="4"/>
-        <v>577.21566489999998</v>
-      </c>
-      <c r="G18" s="17">
-        <f t="shared" si="3"/>
-        <v>0.57721566489999998</v>
-      </c>
-      <c r="H18" s="21">
-        <f t="shared" si="4"/>
-        <v>577.21566489999998</v>
-      </c>
-      <c r="I18" s="24">
-        <f t="shared" si="3"/>
-        <v>0.57721566489999998</v>
-      </c>
-      <c r="J18" s="27">
-        <f t="shared" si="7"/>
-        <v>37090</v>
-      </c>
-      <c r="K18" s="30">
-        <f t="shared" si="7"/>
-        <v>37090</v>
-      </c>
-      <c r="L18" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Wed</v>
-      </c>
-      <c r="M18" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N18" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="5">
-        <f xml:space="preserve"> LN(2)</f>
-        <v>0.69314718055994529</v>
-      </c>
-      <c r="D19" s="9">
-        <f t="shared" si="3"/>
-        <v>0.69314718055994529</v>
-      </c>
-      <c r="E19" s="12">
-        <f t="shared" si="3"/>
-        <v>0.69314718055994529</v>
-      </c>
-      <c r="F19" s="15">
-        <f t="shared" si="4"/>
-        <v>693.14718055994524</v>
-      </c>
-      <c r="G19" s="17">
-        <f t="shared" si="3"/>
-        <v>0.69314718055994529</v>
-      </c>
-      <c r="H19" s="21">
-        <f t="shared" si="4"/>
-        <v>693.14718055994524</v>
-      </c>
-      <c r="I19" s="24">
-        <f t="shared" si="3"/>
-        <v>0.69314718055994529</v>
-      </c>
-      <c r="J19" s="27">
-        <f t="shared" si="7"/>
-        <v>37155</v>
-      </c>
-      <c r="K19" s="30">
-        <f t="shared" si="7"/>
-        <v>37155</v>
-      </c>
-      <c r="L19" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Fri</v>
-      </c>
-      <c r="M19" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N19" s="36" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="1" t="b">
-        <f xml:space="preserve"> TRUE</f>
-        <v>1</v>
-      </c>
-      <c r="C20" s="5">
-        <f>LOG10(5)</f>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="D20" s="9">
-        <f t="shared" si="3"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="E20" s="12">
-        <f t="shared" si="3"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="F20" s="15">
-        <f t="shared" si="4"/>
-        <v>698.97000433601886</v>
-      </c>
-      <c r="G20" s="17">
-        <f t="shared" si="3"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="H20" s="21">
-        <f t="shared" si="4"/>
-        <v>698.97000433601886</v>
-      </c>
-      <c r="I20" s="24">
-        <f t="shared" si="3"/>
-        <v>0.69897000433601886</v>
-      </c>
-      <c r="J20" s="27">
-        <f t="shared" si="7"/>
-        <v>37155</v>
-      </c>
-      <c r="K20" s="30">
-        <f t="shared" si="7"/>
-        <v>37155</v>
-      </c>
-      <c r="L20" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Fri</v>
-      </c>
-      <c r="M20" s="33">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N20" s="36" t="s">
-        <v>23</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="B5:O5" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
-  <headerFooter>
-    <oddHeader>&amp;L&amp;F&amp;CU//FOUO&amp;R&amp;A</oddHeader>
-    <oddFooter>&amp;Lprinted: &amp;D&amp;CU//FOUO&amp;Rpage &amp;P of &amp;N</oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
data > xl > ml-4350-notes-CY25-Q3.xlsx: new filename entered: "s5c_ts_fourier.qmd", with dependency "spectrum_helpers.R".
</commit_message>
<xml_diff>
--- a/data/xl/ml-4350-notes-CY25-Q3a.xlsx
+++ b/data/xl/ml-4350-notes-CY25-Q3a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ca9ccbbb0bd9c947/Documents/GitHub/eda_4350/data/xl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="350" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A24934D8-4E3C-431D-A2EB-D2C63CE03641}"/>
+  <xr:revisionPtr revIDLastSave="358" documentId="8_{BE919223-632E-4CA3-A135-7A7680007E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C2D0162-445E-4F9A-A447-2AE85DBD215C}"/>
   <bookViews>
-    <workbookView xWindow="786" yWindow="138" windowWidth="18858" windowHeight="11136" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="786" yWindow="138" windowWidth="18858" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="index" sheetId="2" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="469">
   <si>
     <t>tag</t>
   </si>
@@ -1465,6 +1465,15 @@
   </si>
   <si>
     <t>I</t>
+  </si>
+  <si>
+    <t>s5c</t>
+  </si>
+  <si>
+    <t>ts_fourier</t>
+  </si>
+  <si>
+    <t>Time Series Spectrum Analysis</t>
   </si>
 </sst>
 </file>
@@ -2301,7 +2310,7 @@
         <v>422</v>
       </c>
       <c r="D8" s="49">
-        <v>45840</v>
+        <v>45854</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>43</v>
@@ -3991,7 +4000,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3225F869-A66F-4DF1-AB64-655834E8B245}">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="1.68359375" style="1" customWidth="1"/>
@@ -4348,7 +4357,7 @@
         <v>403</v>
       </c>
       <c r="E15" s="1" t="str">
-        <f t="shared" ref="E15:E18" si="1" xml:space="preserve"> $C15 &amp; "_" &amp; $D15</f>
+        <f t="shared" ref="E15:E19" si="1" xml:space="preserve"> $C15 &amp; "_" &amp; $D15</f>
         <v>s5b_ts_forecast</v>
       </c>
       <c r="F15" s="1" t="s">
@@ -4358,7 +4367,7 @@
         <v>419</v>
       </c>
       <c r="H15" s="1" t="str">
-        <f t="shared" ref="H15:I15" si="2">H14</f>
+        <f t="shared" ref="H15:I16" si="2">H14</f>
         <v>gen_ds_tbl.R</v>
       </c>
       <c r="I15" s="1" t="str">
@@ -4374,26 +4383,27 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="B16" s="45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>416</v>
+        <v>466</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>404</v>
+        <v>467</v>
       </c>
       <c r="E16" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>s6a_topic_review</v>
+        <v>s5c_ts_fourier</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>365</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>426</v>
+        <v>468</v>
+      </c>
+      <c r="H16" s="1" t="str">
+        <f xml:space="preserve"> "spectrum_helpers.R"</f>
+        <v>spectrum_helpers.R</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>435</v>
@@ -4407,20 +4417,20 @@
         <v>6</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E17" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>s6b_discussion</v>
+        <v>s6a_topic_review</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>365</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>426</v>
@@ -4434,31 +4444,61 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>425</v>
+        <v>405</v>
       </c>
       <c r="E18" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>xtra_Dirichlet_dstn</v>
+        <v>s6b_discussion</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>365</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>426</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="45">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="E19" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>xtra_Dirichlet_dstn</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="J19" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="L19" s="1" t="s">
         <v>433</v>
       </c>
     </row>

</xml_diff>